<commit_message>
feat: Implement vectorized Monte Carlo simulation for NBA game outcomes, update README to reflect 1M iterations, and add system overview documentation.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-11.xlsx
+++ b/results/nba_predictions_2025-12-11.xlsx
@@ -568,10 +568,10 @@
         <v>24.32</v>
       </c>
       <c r="F2" t="n">
-        <v>58.23</v>
+        <v>57.67</v>
       </c>
       <c r="G2" t="n">
-        <v>41.77</v>
+        <v>42.33</v>
       </c>
       <c r="H2" t="n">
         <v>0.54</v>
@@ -653,10 +653,10 @@
         <v>75.27</v>
       </c>
       <c r="F3" t="n">
-        <v>54.76</v>
+        <v>54.78</v>
       </c>
       <c r="G3" t="n">
-        <v>45.24</v>
+        <v>45.22</v>
       </c>
       <c r="H3" t="n">
         <v>-0.42</v>
@@ -738,10 +738,10 @@
         <v>84</v>
       </c>
       <c r="F4" t="n">
-        <v>54.78</v>
+        <v>54.92</v>
       </c>
       <c r="G4" t="n">
-        <v>45.22</v>
+        <v>45.08</v>
       </c>
       <c r="H4" t="n">
         <v>-0.7</v>
@@ -823,10 +823,10 @@
         <v>75.27</v>
       </c>
       <c r="F5" t="n">
-        <v>55.24</v>
+        <v>55.29</v>
       </c>
       <c r="G5" t="n">
-        <v>44.76</v>
+        <v>44.71</v>
       </c>
       <c r="H5" t="n">
         <v>-0.52</v>

</xml_diff>

<commit_message>
feat: Introduce CLI, ML retraining, and health check scripts, enhance financial risk management, and update orchestrator to v21.5 after forensic audit.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-11.xlsx
+++ b/results/nba_predictions_2025-12-11.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>75.68000000000001</v>
+        <v>52.59</v>
       </c>
       <c r="E2" t="n">
-        <v>24.32</v>
+        <v>47.41</v>
       </c>
       <c r="F2" t="n">
-        <v>57.67</v>
+        <v>57.89</v>
       </c>
       <c r="G2" t="n">
-        <v>42.33</v>
+        <v>42.11</v>
       </c>
       <c r="H2" t="n">
         <v>0.54</v>
@@ -586,14 +586,14 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>1.831199428709592</v>
+        <v>1.831195315604405</v>
       </c>
       <c r="M2" t="n">
-        <v>2.203080711391326</v>
+        <v>2.203086664742387</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,10 +608,10 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>75.7</v>
+        <v>52.6</v>
       </c>
       <c r="S2" t="n">
-        <v>24.3</v>
+        <v>47.4</v>
       </c>
       <c r="T2" t="n">
         <v>221.5</v>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>15.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>24.73</v>
+        <v>14.83</v>
       </c>
       <c r="E3" t="n">
-        <v>75.27</v>
+        <v>85.17</v>
       </c>
       <c r="F3" t="n">
-        <v>54.78</v>
+        <v>54.74</v>
       </c>
       <c r="G3" t="n">
-        <v>45.22</v>
+        <v>45.26</v>
       </c>
       <c r="H3" t="n">
         <v>-0.42</v>
@@ -693,10 +693,10 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>24.7</v>
+        <v>14.8</v>
       </c>
       <c r="S3" t="n">
-        <v>75.3</v>
+        <v>85.2</v>
       </c>
       <c r="T3" t="n">
         <v>228.3</v>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>-15.2</v>
+        <v>-21.1</v>
       </c>
     </row>
     <row r="4">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>14.31</v>
       </c>
       <c r="E4" t="n">
-        <v>84</v>
+        <v>85.69</v>
       </c>
       <c r="F4" t="n">
-        <v>54.92</v>
+        <v>55.22</v>
       </c>
       <c r="G4" t="n">
-        <v>45.08</v>
+        <v>44.78</v>
       </c>
       <c r="H4" t="n">
         <v>-0.7</v>
@@ -756,10 +756,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1.89333406670255</v>
+        <v>1.893260181622106</v>
       </c>
       <c r="M4" t="n">
-        <v>2.119402066117519</v>
+        <v>2.11949465628711</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -778,10 +778,10 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>16</v>
+        <v>14.3</v>
       </c>
       <c r="S4" t="n">
-        <v>84</v>
+        <v>85.7</v>
       </c>
       <c r="T4" t="n">
         <v>222.1</v>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>-20.4</v>
+        <v>-21.4</v>
       </c>
     </row>
     <row r="5">
@@ -817,16 +817,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24.73</v>
+        <v>14.83</v>
       </c>
       <c r="E5" t="n">
-        <v>75.27</v>
+        <v>85.17</v>
       </c>
       <c r="F5" t="n">
-        <v>55.29</v>
+        <v>55.25</v>
       </c>
       <c r="G5" t="n">
-        <v>44.71</v>
+        <v>44.75</v>
       </c>
       <c r="H5" t="n">
         <v>-0.52</v>
@@ -841,10 +841,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>1.896290637728825</v>
+        <v>1.896335547175098</v>
       </c>
       <c r="M5" t="n">
-        <v>2.115709523122959</v>
+        <v>2.1156536222976</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -863,10 +863,10 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>24.7</v>
+        <v>14.8</v>
       </c>
       <c r="S5" t="n">
-        <v>75.3</v>
+        <v>85.2</v>
       </c>
       <c r="T5" t="n">
         <v>225.5</v>
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>-15.2</v>
+        <v>-21.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement new ML pipeline modules, data scraping, utility scripts, and MLflow tracking, alongside updates to the orchestrator and web application.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-11.xlsx
+++ b/results/nba_predictions_2025-12-11.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>52.59</v>
+        <v>75.68000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>47.41</v>
+        <v>24.32</v>
       </c>
       <c r="F2" t="n">
-        <v>57.89</v>
+        <v>57.97</v>
       </c>
       <c r="G2" t="n">
-        <v>42.11</v>
+        <v>42.03</v>
       </c>
       <c r="H2" t="n">
         <v>0.54</v>
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,10 +608,10 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>52.6</v>
+        <v>75.7</v>
       </c>
       <c r="S2" t="n">
-        <v>47.4</v>
+        <v>24.3</v>
       </c>
       <c r="T2" t="n">
         <v>221.5</v>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>1.6</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="3">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>14.83</v>
+        <v>15.2</v>
       </c>
       <c r="E3" t="n">
-        <v>85.17</v>
+        <v>84.8</v>
       </c>
       <c r="F3" t="n">
-        <v>54.74</v>
+        <v>54.72</v>
       </c>
       <c r="G3" t="n">
-        <v>45.26</v>
+        <v>45.28</v>
       </c>
       <c r="H3" t="n">
         <v>-0.42</v>
@@ -693,10 +693,10 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="S3" t="n">
-        <v>85.2</v>
+        <v>84.8</v>
       </c>
       <c r="T3" t="n">
         <v>228.3</v>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>-21.1</v>
+        <v>-20.9</v>
       </c>
     </row>
     <row r="4">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>14.31</v>
+        <v>15.2</v>
       </c>
       <c r="E4" t="n">
-        <v>85.69</v>
+        <v>84.8</v>
       </c>
       <c r="F4" t="n">
-        <v>55.22</v>
+        <v>55.17</v>
       </c>
       <c r="G4" t="n">
-        <v>44.78</v>
+        <v>44.83</v>
       </c>
       <c r="H4" t="n">
         <v>-0.7</v>
@@ -778,10 +778,10 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>14.3</v>
+        <v>15.2</v>
       </c>
       <c r="S4" t="n">
-        <v>85.7</v>
+        <v>84.8</v>
       </c>
       <c r="T4" t="n">
         <v>222.1</v>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>-21.4</v>
+        <v>-20.9</v>
       </c>
     </row>
     <row r="5">
@@ -817,16 +817,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14.83</v>
+        <v>15.2</v>
       </c>
       <c r="E5" t="n">
-        <v>85.17</v>
+        <v>84.8</v>
       </c>
       <c r="F5" t="n">
-        <v>55.25</v>
+        <v>55.28</v>
       </c>
       <c r="G5" t="n">
-        <v>44.75</v>
+        <v>44.72</v>
       </c>
       <c r="H5" t="n">
         <v>-0.52</v>
@@ -863,10 +863,10 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="S5" t="n">
-        <v>85.2</v>
+        <v>84.8</v>
       </c>
       <c r="T5" t="n">
         <v>225.5</v>
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>-21.1</v>
+        <v>-20.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>